<commit_message>
median waretfall plots based
</commit_message>
<xml_diff>
--- a/heatmap_drug_waterfall_summary_tables.xlsx
+++ b/heatmap_drug_waterfall_summary_tables.xlsx
@@ -27,43 +27,55 @@
     <t xml:space="preserve">aPD1+ Venetoclax (Bcl-2)</t>
   </si>
   <si>
+    <t xml:space="preserve">Panobinostat (HDAC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aPD1+ NFkB Act Inhib (NFkB)</t>
+  </si>
+  <si>
     <t xml:space="preserve">aPD1+ Panobinostat (HDAC)</t>
   </si>
   <si>
     <t xml:space="preserve">NFkB Act Inhib (NFkB)</t>
   </si>
   <si>
-    <t xml:space="preserve">aPD1+ NFkB Act Inhib (NFkB)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Panobinostat (HDAC)</t>
+    <t xml:space="preserve">aPD1+ Trametinib (MEK)</t>
   </si>
   <si>
     <t xml:space="preserve">Trametinib (MEK)</t>
   </si>
   <si>
-    <t xml:space="preserve">aPD1+ Trametinib (MEK)</t>
-  </si>
-  <si>
     <t xml:space="preserve">JQ1 (BRD4)</t>
   </si>
   <si>
+    <t xml:space="preserve">Palbociclib (CDK46)</t>
+  </si>
+  <si>
     <t xml:space="preserve">aPD1+ Dasatinib (SFKs)</t>
   </si>
   <si>
     <t xml:space="preserve">aPD1+ MK-2206 (AKT)</t>
   </si>
   <si>
-    <t xml:space="preserve">Palbociclib (CDK46)</t>
+    <t xml:space="preserve">aPD1+ Palbociclib (CDK46)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aPD1+ CYT387 (JAK)</t>
   </si>
   <si>
     <t xml:space="preserve">MK-2206 (AKT)</t>
   </si>
   <si>
-    <t xml:space="preserve">aPD1+ Palbociclib (CDK46)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aPD1+ CYT387 (JAK)</t>
+    <t xml:space="preserve">aPD1+ PD173074 (FGFR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CYT387 (JAK)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GW-2580 (CSFIR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dasatinib (SFKs)</t>
   </si>
   <si>
     <t xml:space="preserve">Sorafenib (FLT3)</t>
@@ -72,64 +84,52 @@
     <t xml:space="preserve">aPD1+ JQ1 (BRD4)</t>
   </si>
   <si>
-    <t xml:space="preserve">Dasatinib (SFKs)</t>
+    <t xml:space="preserve">aPD1+ Olaparib (PARP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NVP-TAE684 (ALK/MET)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aPD1+ Sorafenib (FLT3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PD173074 (FGFR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aPD1+ Ibrutinib (TEC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doramapimod (p38)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Olaparib (PARP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aPD1+ Doramapimod (p38)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEZ235 (PI3K/mTOR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aPD1+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aPD1+ GW-2580 (CSFIR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aPD1+ BEZ235 (PI3K/mTOR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entospletinib (SYK)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aPD1+ Entospletinib (SYK)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aPD1+ NVP-TAE684 (ALK/MET)</t>
   </si>
   <si>
     <t xml:space="preserve">Ibrutinib (TEC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GW-2580 (CSFIR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aPD1+ PD173074 (FGFR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CYT387 (JAK)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aPD1+ Sorafenib (FLT3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Doramapimod (p38)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aPD1+ Olaparib (PARP)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aPD1+ Doramapimod (p38)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PD173074 (FGFR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entospletinib (SYK)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Olaparib (PARP)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aPD1+ BEZ235 (PI3K/mTOR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aPD1+ NVP-TAE684 (ALK/MET)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aPD1+ GW-2580 (CSFIR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEZ235 (PI3K/mTOR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NVP-TAE684 (ALK/MET)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aPD1+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aPD1+ Ibrutinib (TEC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aPD1+ Entospletinib (SYK)</t>
   </si>
 </sst>
 </file>
@@ -471,7 +471,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>2.29722589082353</v>
+        <v>2.48204238</v>
       </c>
     </row>
     <row r="3">
@@ -479,7 +479,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>1.6220678113125</v>
+        <v>1.6075138245</v>
       </c>
     </row>
     <row r="4">
@@ -487,7 +487,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>1.10698314211765</v>
+        <v>1.02963495</v>
       </c>
     </row>
     <row r="5">
@@ -495,7 +495,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>1.06868956135294</v>
+        <v>1.00458187</v>
       </c>
     </row>
     <row r="6">
@@ -503,7 +503,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>1.03361343676471</v>
+        <v>0.91326132</v>
       </c>
     </row>
     <row r="7">
@@ -511,7 +511,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>0.947776988882353</v>
+        <v>0.788785108</v>
       </c>
     </row>
     <row r="8">
@@ -519,7 +519,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.462984453411765</v>
+        <v>0.20238414</v>
       </c>
     </row>
     <row r="9">
@@ -527,7 +527,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="n">
-        <v>0.275189938294118</v>
+        <v>0.16681658</v>
       </c>
     </row>
     <row r="10">
@@ -535,7 +535,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="n">
-        <v>0.0577597201764706</v>
+        <v>0.097499532</v>
       </c>
     </row>
     <row r="11">
@@ -543,7 +543,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="n">
-        <v>0.0141898535294118</v>
+        <v>-0.0885361</v>
       </c>
     </row>
     <row r="12">
@@ -551,7 +551,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="n">
-        <v>0.00611084117647057</v>
+        <v>-0.1350815</v>
       </c>
     </row>
     <row r="13">
@@ -559,7 +559,7 @@
         <v>13</v>
       </c>
       <c r="B13" t="n">
-        <v>0.00112308517647058</v>
+        <v>-0.1523187</v>
       </c>
     </row>
     <row r="14">
@@ -567,7 +567,7 @@
         <v>14</v>
       </c>
       <c r="B14" t="n">
-        <v>-0.0709343619411765</v>
+        <v>-0.1578458</v>
       </c>
     </row>
     <row r="15">
@@ -575,7 +575,7 @@
         <v>15</v>
       </c>
       <c r="B15" t="n">
-        <v>-0.0772583511176471</v>
+        <v>-0.22591395</v>
       </c>
     </row>
     <row r="16">
@@ -583,7 +583,7 @@
         <v>16</v>
       </c>
       <c r="B16" t="n">
-        <v>-0.107828246823529</v>
+        <v>-0.2466787</v>
       </c>
     </row>
     <row r="17">
@@ -591,7 +591,7 @@
         <v>17</v>
       </c>
       <c r="B17" t="n">
-        <v>-0.115211741117647</v>
+        <v>-0.25783026</v>
       </c>
     </row>
     <row r="18">
@@ -599,7 +599,7 @@
         <v>18</v>
       </c>
       <c r="B18" t="n">
-        <v>-0.197088315352941</v>
+        <v>-0.26506309</v>
       </c>
     </row>
     <row r="19">
@@ -607,7 +607,7 @@
         <v>19</v>
       </c>
       <c r="B19" t="n">
-        <v>-0.232109615941176</v>
+        <v>-0.27727382</v>
       </c>
     </row>
     <row r="20">
@@ -615,7 +615,7 @@
         <v>20</v>
       </c>
       <c r="B20" t="n">
-        <v>-0.261458047882353</v>
+        <v>-0.3173918</v>
       </c>
     </row>
     <row r="21">
@@ -623,7 +623,7 @@
         <v>21</v>
       </c>
       <c r="B21" t="n">
-        <v>-0.2624981784375</v>
+        <v>-0.326600256</v>
       </c>
     </row>
     <row r="22">
@@ -631,7 +631,7 @@
         <v>22</v>
       </c>
       <c r="B22" t="n">
-        <v>-0.276152915823529</v>
+        <v>-0.337426713</v>
       </c>
     </row>
     <row r="23">
@@ -639,7 +639,7 @@
         <v>23</v>
       </c>
       <c r="B23" t="n">
-        <v>-0.279701341058824</v>
+        <v>-0.388472356</v>
       </c>
     </row>
     <row r="24">
@@ -647,7 +647,7 @@
         <v>24</v>
       </c>
       <c r="B24" t="n">
-        <v>-0.280167213294118</v>
+        <v>-0.38987498</v>
       </c>
     </row>
     <row r="25">
@@ -655,7 +655,7 @@
         <v>25</v>
       </c>
       <c r="B25" t="n">
-        <v>-0.302021017</v>
+        <v>-0.458466105</v>
       </c>
     </row>
     <row r="26">
@@ -663,7 +663,7 @@
         <v>26</v>
       </c>
       <c r="B26" t="n">
-        <v>-0.338927096705882</v>
+        <v>-0.493642367</v>
       </c>
     </row>
     <row r="27">
@@ -671,7 +671,7 @@
         <v>27</v>
       </c>
       <c r="B27" t="n">
-        <v>-0.363364917294118</v>
+        <v>-0.50680532</v>
       </c>
     </row>
     <row r="28">
@@ -679,7 +679,7 @@
         <v>28</v>
       </c>
       <c r="B28" t="n">
-        <v>-0.442824605</v>
+        <v>-0.507113505</v>
       </c>
     </row>
     <row r="29">
@@ -687,7 +687,7 @@
         <v>29</v>
       </c>
       <c r="B29" t="n">
-        <v>-0.443069745470588</v>
+        <v>-0.517890415</v>
       </c>
     </row>
     <row r="30">
@@ -695,7 +695,7 @@
         <v>30</v>
       </c>
       <c r="B30" t="n">
-        <v>-0.448105499294118</v>
+        <v>-0.531361553</v>
       </c>
     </row>
     <row r="31">
@@ -703,7 +703,7 @@
         <v>31</v>
       </c>
       <c r="B31" t="n">
-        <v>-0.477735384941176</v>
+        <v>-0.5506315</v>
       </c>
     </row>
     <row r="32">
@@ -711,7 +711,7 @@
         <v>32</v>
       </c>
       <c r="B32" t="n">
-        <v>-0.4809547591875</v>
+        <v>-0.560998057</v>
       </c>
     </row>
     <row r="33">
@@ -719,7 +719,7 @@
         <v>33</v>
       </c>
       <c r="B33" t="n">
-        <v>-0.489872150125</v>
+        <v>-0.569134315</v>
       </c>
     </row>
     <row r="34">
@@ -727,7 +727,7 @@
         <v>34</v>
       </c>
       <c r="B34" t="n">
-        <v>-0.498039126764706</v>
+        <v>-0.57337917</v>
       </c>
     </row>
     <row r="35">
@@ -735,7 +735,7 @@
         <v>35</v>
       </c>
       <c r="B35" t="n">
-        <v>-0.511948245529412</v>
+        <v>-0.5768096</v>
       </c>
     </row>
     <row r="36">
@@ -743,7 +743,7 @@
         <v>36</v>
       </c>
       <c r="B36" t="n">
-        <v>-0.559824254</v>
+        <v>-0.59406356</v>
       </c>
     </row>
     <row r="37">
@@ -751,7 +751,7 @@
         <v>37</v>
       </c>
       <c r="B37" t="n">
-        <v>-0.610468722411765</v>
+        <v>-0.59581988</v>
       </c>
     </row>
     <row r="38">
@@ -759,7 +759,7 @@
         <v>38</v>
       </c>
       <c r="B38" t="n">
-        <v>-0.743283644588235</v>
+        <v>-0.607968621</v>
       </c>
     </row>
   </sheetData>
@@ -783,298 +783,298 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B2" t="n">
-        <v>1.68181162960514</v>
+        <v>1.27416023862891</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B3" t="n">
-        <v>1.25722565196841</v>
+        <v>0.697678960147801</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B4" t="n">
-        <v>0.719087490556125</v>
+        <v>0.679293754119638</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="B5" t="n">
-        <v>0.486131327297147</v>
+        <v>0.3104472851</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="B6" t="n">
-        <v>0.341253991015718</v>
+        <v>0.293659162703544</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B7" t="n">
-        <v>0.219085139313304</v>
+        <v>0.146385889857151</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="B8" t="n">
-        <v>0.201431014237564</v>
+        <v>0.0536709225592455</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="B9" t="n">
-        <v>0.175618499811771</v>
+        <v>0.0348033522761322</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="B10" t="n">
-        <v>0.120226678304647</v>
+        <v>0.0270081164726414</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="B11" t="n">
-        <v>0.120072562439965</v>
+        <v>-0.0155816566681302</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="B12" t="n">
-        <v>0.116362036348629</v>
+        <v>-0.0725747026417</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B13" t="n">
-        <v>0.107184688941079</v>
+        <v>-0.0843559995</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B14" t="n">
-        <v>0.107009849814383</v>
+        <v>-0.088255946953118</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="B15" t="n">
-        <v>0.094693319925973</v>
+        <v>-0.0987264244532232</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="B16" t="n">
-        <v>0.0493527722724307</v>
+        <v>-0.1134566265</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B17" t="n">
-        <v>0.0353747222072831</v>
+        <v>-0.1165902026</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="B18" t="n">
-        <v>0.0339357585759499</v>
+        <v>-0.139623976</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B19" t="n">
-        <v>0.011368768460062</v>
+        <v>-0.155225094323573</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="B20" t="n">
-        <v>0.00372485424365414</v>
+        <v>-0.16226705753647</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="B21" t="n">
-        <v>-0.0395323120977915</v>
+        <v>-0.2014967935</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="B22" t="n">
-        <v>-0.0665871611572895</v>
+        <v>-0.221717528561506</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B23" t="n">
-        <v>-0.126198142388506</v>
+        <v>-0.222022137990056</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="B24" t="n">
-        <v>-0.175519734532497</v>
+        <v>-0.22277405979276</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B25" t="n">
-        <v>-0.226159113296606</v>
+        <v>-0.296571943</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B26" t="n">
-        <v>-0.230468596851979</v>
+        <v>-0.311596977832993</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="B27" t="n">
-        <v>-0.245860761570373</v>
+        <v>-0.35309025</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="B28" t="n">
-        <v>-0.253057345948099</v>
+        <v>-0.367432979469388</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="B29" t="n">
-        <v>-0.283050580249457</v>
+        <v>-0.370676228617759</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="B30" t="n">
-        <v>-0.309377245102735</v>
+        <v>-0.417942228</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B31" t="n">
-        <v>-0.329411975749373</v>
+        <v>-0.444739709711049</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B32" t="n">
-        <v>-0.437795839284446</v>
+        <v>-0.492740965689505</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B33" t="n">
-        <v>-0.517308265198081</v>
+        <v>-0.558094886093589</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B34" t="n">
-        <v>-0.527888974190665</v>
+        <v>-0.624614101179384</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="B35" t="n">
-        <v>-0.586269754685875</v>
+        <v>-0.641530955493996</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B36" t="n">
-        <v>-0.606756470151614</v>
+        <v>-0.643875482038198</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B37" t="n">
-        <v>-0.666106981024532</v>
+        <v>-0.72360254836672</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B38" t="n">
-        <v>-0.721274111269177</v>
+        <v>-0.725517391</v>
       </c>
     </row>
   </sheetData>

</xml_diff>